<commit_message>
subida de fichas tecnicas
</commit_message>
<xml_diff>
--- a/datos_samm/Fichas_Drive.xlsx
+++ b/datos_samm/Fichas_Drive.xlsx
@@ -1,23 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion rupBuild="9303" lowestEdited="5" lastEdited="5" appName="xl"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Analista Contable\Desktop\Dino-erp\datos_samm\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7008B01-5678-49A4-9C5E-5D70DB54DB25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet r:id="rId1" sheetId="1" name="Hoja 1"/>
+    <sheet name="Hoja 1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Hoja 1'!$A$1:$C$232</definedName>
   </definedNames>
-  <calcPr fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="696" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="726" uniqueCount="489">
   <si>
     <t>Nombre_Archivo</t>
   </si>
@@ -1424,14 +1430,73 @@
   </si>
   <si>
     <t>https://docs.google.com/spreadsheets/d/1HrFhxk3gOMDO3xHEh0CM7q1uJrK3nIWl/edit?usp=drivesdk&amp;ouid=104727614470399304054&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Ficha Tecnica FE0 - 440.xlsx</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1IOBbku5vszPNU9qHTMlC_XRTVfwnuxEC/edit?usp=drivesdk&amp;ouid=104727614470399304054&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Ficha Tecnica FD9 - 439.xlsx</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1uiVpxREw-ttPpRp9PfUhG0s4V96Xwz55/edit?usp=drivesdk&amp;ouid=104727614470399304054&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Ficha Tecnica FD8 - 438.xlsx</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1CPLVwERB6Kd3KmIy1zsBPKItAlkV8nVw/edit?usp=drivesdk&amp;ouid=104727614470399304054&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Ficha Tecnica FD7 - 437.xlsx</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1sH_1FxMFXIxptQUeHrQ3Xf9RNhcUUaA2/edit?usp=drivesdk&amp;ouid=104727614470399304054&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Ficha Tecnica FD6 - 436.xlsx</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/15p9AxqY_zu2BHJlFH94ROlk6hOnomkdY/edit?usp=drivesdk&amp;ouid=104727614470399304054&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Ficha Tecnica FD5 - 435.xlsx</t>
+  </si>
+  <si>
+    <t>Ficha Tecnica FD4 - 434.xlsx</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1YkvHpj1w4Suoe-Xc0luKitY8v30QzBqz/edit?usp=drivesdk&amp;ouid=104727614470399304054&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Ficha Tecnica FD3 - 433.xlsx</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1yCkied80ubvOqDcMC3NT5GIrhtOjs4jG/edit?usp=drivesdk&amp;ouid=104727614470399304054&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Ficha Tecnica FD2 - 432.xlsx</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1g_t_bb3RFIteJKn-bb3Akyj4aY2trNmp/edit?usp=drivesdk&amp;ouid=104727614470399304054&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>Ficha Tecnica FD2 - 430.xlsx</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1Lwi_kpumF9NuvqhOcGEaq_NOL2g8RnAT/edit?usp=drivesdk&amp;ouid=104727614470399304054&amp;rtpof=true&amp;sd=true</t>
+  </si>
+  <si>
+    <t>https://docs.google.com/spreadsheets/d/1YwpQy_qUdBu84QnyJWRyoXGChdIS-Dtd/edit?gid=215926301#gid=215926301</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" mc:Ignorable="x14ac">
-  <numFmts count="0"/>
-  <fonts count="4" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1448,16 +1513,23 @@
     <font>
       <u/>
       <sz val="10"/>
-      <color rgb="FF0000ff"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <u/>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -1485,52 +1557,60 @@
     </border>
     <border>
       <left style="medium">
-        <color rgb="FFcccccc"/>
+        <color rgb="FFCCCCCC"/>
       </left>
       <right style="medium">
-        <color rgb="FFcccccc"/>
+        <color rgb="FFCCCCCC"/>
       </right>
       <top style="medium">
-        <color rgb="FFcccccc"/>
+        <color rgb="FFCCCCCC"/>
       </top>
       <bottom style="medium">
-        <color rgb="FFcccccc"/>
+        <color rgb="FFCCCCCC"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="2" applyBorder="1" fontId="3" applyFont="1" fillId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
-    </xf>
   </cellXfs>
-  <cellStyles count="1">
-    <cellStyle xfId="0" builtinId="0" name="Normal"/>
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
-    <ext uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14ac:slicerStyles xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" defaultSlicerStyle="SlicerStyleLight1"/>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -1541,10 +1621,10 @@
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr lastClr="000000" val="windowText"/>
+        <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr lastClr="FFFFFF" val="window"/>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="000000"/>
@@ -1582,71 +1662,71 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Times New Roman" script="Arab"/>
-        <a:font typeface="Times New Roman" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="MoolBoran" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Times New Roman" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font typeface="ＭＳ Ｐゴシック" script="Jpan"/>
-        <a:font typeface="맑은 고딕" script="Hang"/>
-        <a:font typeface="宋体" script="Hans"/>
-        <a:font typeface="新細明體" script="Hant"/>
-        <a:font typeface="Arial" script="Arab"/>
-        <a:font typeface="Arial" script="Hebr"/>
-        <a:font typeface="Tahoma" script="Thai"/>
-        <a:font typeface="Nyala" script="Ethi"/>
-        <a:font typeface="Vrinda" script="Beng"/>
-        <a:font typeface="Shruti" script="Gujr"/>
-        <a:font typeface="DaunPenh" script="Khmr"/>
-        <a:font typeface="Tunga" script="Knda"/>
-        <a:font typeface="Raavi" script="Guru"/>
-        <a:font typeface="Euphemia" script="Cans"/>
-        <a:font typeface="Plantagenet Cherokee" script="Cher"/>
-        <a:font typeface="Microsoft Yi Baiti" script="Yiii"/>
-        <a:font typeface="Microsoft Himalaya" script="Tibt"/>
-        <a:font typeface="MV Boli" script="Thaa"/>
-        <a:font typeface="Mangal" script="Deva"/>
-        <a:font typeface="Gautami" script="Telu"/>
-        <a:font typeface="Latha" script="Taml"/>
-        <a:font typeface="Estrangelo Edessa" script="Syrc"/>
-        <a:font typeface="Kalinga" script="Orya"/>
-        <a:font typeface="Kartika" script="Mlym"/>
-        <a:font typeface="DokChampa" script="Laoo"/>
-        <a:font typeface="Iskoola Pota" script="Sinh"/>
-        <a:font typeface="Mongolian Baiti" script="Mong"/>
-        <a:font typeface="Arial" script="Viet"/>
-        <a:font typeface="Microsoft Uighur" script="Uigh"/>
-        <a:font typeface="Sylfaen" script="Geor"/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -1674,7 +1754,7 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
@@ -1697,11 +1777,11 @@
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin scaled="1" ang="16200000"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="9525">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr">
               <a:shade val="9500"/>
@@ -1710,13 +1790,13 @@
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="25400">
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
         </a:ln>
-        <a:ln algn="ctr" cmpd="sng" cap="flat" w="38100">
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -1726,7 +1806,7 @@
       <a:effectStyleLst>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="38000"/>
               </a:srgbClr>
@@ -1735,7 +1815,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1744,7 +1824,7 @@
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw dir="5400000" rotWithShape="0" dist="23000" blurRad="40000">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
                 <a:alpha val="35000"/>
               </a:srgbClr>
@@ -1752,10 +1832,10 @@
           </a:effectLst>
           <a:scene3d>
             <a:camera prst="orthographicFront">
-              <a:rot rev="0" lon="0" lat="0"/>
+              <a:rot lat="0" lon="0" rev="0"/>
             </a:camera>
-            <a:lightRig dir="t" rig="threePt">
-              <a:rot rev="1200000" lon="0" lat="0"/>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
             </a:lightRig>
           </a:scene3d>
           <a:sp3d>
@@ -1820,19 +1900,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:C232"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:C242"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="6" width="35.71928571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="6" width="171.29071428571427" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="6" width="32.43357142857143" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" width="35.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="171.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="32.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75" hidden="1">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1843,7 +1923,7 @@
         <v>2</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75" hidden="1">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -1854,7 +1934,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75" hidden="1">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
@@ -1865,7 +1945,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75" hidden="1">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
@@ -1876,7 +1956,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75" hidden="1">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>10</v>
       </c>
@@ -1887,7 +1967,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75" hidden="1">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
@@ -1898,7 +1978,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75" hidden="1">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -1909,7 +1989,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75" hidden="1">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
@@ -1920,7 +2000,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75" hidden="1">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>18</v>
       </c>
@@ -1931,7 +2011,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75" hidden="1">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>20</v>
       </c>
@@ -1942,7 +2022,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75" hidden="1">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>22</v>
       </c>
@@ -1953,7 +2033,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="18.75" hidden="1">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
@@ -1964,7 +2044,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="13" customHeight="1" ht="18.75" hidden="1">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>26</v>
       </c>
@@ -1975,7 +2055,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="14" customHeight="1" ht="18.75" hidden="1">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>28</v>
       </c>
@@ -1986,7 +2066,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="15" customHeight="1" ht="18.75" hidden="1">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>30</v>
       </c>
@@ -1997,7 +2077,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="16" customHeight="1" ht="18.75" hidden="1">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>32</v>
       </c>
@@ -2008,7 +2088,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="17" customHeight="1" ht="18.75" hidden="1">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>34</v>
       </c>
@@ -2019,7 +2099,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="18" customHeight="1" ht="18.75" hidden="1">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>36</v>
       </c>
@@ -2030,7 +2110,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="19" customHeight="1" ht="18.75" hidden="1">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>38</v>
       </c>
@@ -2041,7 +2121,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="20" customHeight="1" ht="18.75" hidden="1">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>40</v>
       </c>
@@ -2052,7 +2132,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="21" customHeight="1" ht="18.75" hidden="1">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>42</v>
       </c>
@@ -2063,7 +2143,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="22" customHeight="1" ht="18.75" hidden="1">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>44</v>
       </c>
@@ -2074,7 +2154,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="23" customHeight="1" ht="18.75" hidden="1">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>46</v>
       </c>
@@ -2085,7 +2165,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="24" customHeight="1" ht="18.75" hidden="1">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>48</v>
       </c>
@@ -2096,7 +2176,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="25" customHeight="1" ht="18.75" hidden="1">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>50</v>
       </c>
@@ -2107,7 +2187,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="26" customHeight="1" ht="18.75" hidden="1">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>52</v>
       </c>
@@ -2118,7 +2198,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="27" customHeight="1" ht="18.75" hidden="1">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>54</v>
       </c>
@@ -2129,7 +2209,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="28" customHeight="1" ht="18.75" hidden="1">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>56</v>
       </c>
@@ -2140,7 +2220,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="29" customHeight="1" ht="18.75" hidden="1">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>58</v>
       </c>
@@ -2151,7 +2231,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="30" customHeight="1" ht="18.75" hidden="1">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>60</v>
       </c>
@@ -2162,7 +2242,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="31" customHeight="1" ht="18.75" hidden="1">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>62</v>
       </c>
@@ -2173,7 +2253,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="32" customHeight="1" ht="18.75" hidden="1">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>64</v>
       </c>
@@ -2184,7 +2264,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="33" customHeight="1" ht="18.75" hidden="1">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>66</v>
       </c>
@@ -2195,7 +2275,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="34" customHeight="1" ht="18.75" hidden="1">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>68</v>
       </c>
@@ -2206,7 +2286,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="35" customHeight="1" ht="18.75" hidden="1">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>70</v>
       </c>
@@ -2217,7 +2297,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="36" customHeight="1" ht="18.75" hidden="1">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>72</v>
       </c>
@@ -2228,7 +2308,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="37" customHeight="1" ht="18.75" hidden="1">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>74</v>
       </c>
@@ -2239,7 +2319,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="38" customHeight="1" ht="18.75" hidden="1">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>76</v>
       </c>
@@ -2250,7 +2330,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="39" customHeight="1" ht="18.75" hidden="1">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>78</v>
       </c>
@@ -2261,7 +2341,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="40" customHeight="1" ht="18.75" hidden="1">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>80</v>
       </c>
@@ -2272,7 +2352,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="41" customHeight="1" ht="18.75" hidden="1">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>82</v>
       </c>
@@ -2283,7 +2363,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="42" customHeight="1" ht="18.75" hidden="1">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>84</v>
       </c>
@@ -2294,7 +2374,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="43" customHeight="1" ht="18.75" hidden="1">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>86</v>
       </c>
@@ -2305,7 +2385,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="44" customHeight="1" ht="18.75" hidden="1">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>88</v>
       </c>
@@ -2316,7 +2396,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="45" customHeight="1" ht="18.75" hidden="1">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>90</v>
       </c>
@@ -2327,7 +2407,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="46" customHeight="1" ht="18.75" hidden="1">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>92</v>
       </c>
@@ -2338,7 +2418,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="47" customHeight="1" ht="18.75" hidden="1">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>94</v>
       </c>
@@ -2349,7 +2429,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="48" customHeight="1" ht="18.75" hidden="1">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>96</v>
       </c>
@@ -2360,7 +2440,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="49" customHeight="1" ht="18.75" hidden="1">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>98</v>
       </c>
@@ -2371,7 +2451,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="50" customHeight="1" ht="18.75" hidden="1">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>100</v>
       </c>
@@ -2382,7 +2462,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="51" customHeight="1" ht="18.75" hidden="1">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>102</v>
       </c>
@@ -2393,7 +2473,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="52" customHeight="1" ht="18.75" hidden="1">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>104</v>
       </c>
@@ -2404,7 +2484,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="53" customHeight="1" ht="18.75" hidden="1">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>106</v>
       </c>
@@ -2415,7 +2495,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="54" customHeight="1" ht="18.75" hidden="1">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>108</v>
       </c>
@@ -2426,7 +2506,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="55" customHeight="1" ht="18.75" hidden="1">
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
         <v>110</v>
       </c>
@@ -2437,7 +2517,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="56" customHeight="1" ht="18.75" hidden="1">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
         <v>112</v>
       </c>
@@ -2448,7 +2528,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="57" customHeight="1" ht="18.75" hidden="1">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
         <v>114</v>
       </c>
@@ -2459,7 +2539,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="58" customHeight="1" ht="18.75" hidden="1">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
         <v>116</v>
       </c>
@@ -2470,7 +2550,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="59" customHeight="1" ht="18.75" hidden="1">
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A59" s="1" t="s">
         <v>118</v>
       </c>
@@ -2481,7 +2561,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="60" customHeight="1" ht="18.75" hidden="1">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A60" s="1" t="s">
         <v>120</v>
       </c>
@@ -2492,7 +2572,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="61" customHeight="1" ht="18.75" hidden="1">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A61" s="1" t="s">
         <v>122</v>
       </c>
@@ -2503,7 +2583,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="62" customHeight="1" ht="18.75" hidden="1">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A62" s="1" t="s">
         <v>124</v>
       </c>
@@ -2514,7 +2594,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="63" customHeight="1" ht="18.75" hidden="1">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A63" s="1" t="s">
         <v>126</v>
       </c>
@@ -2525,7 +2605,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="64" customHeight="1" ht="18.75" hidden="1">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A64" s="1" t="s">
         <v>128</v>
       </c>
@@ -2536,7 +2616,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="65" customHeight="1" ht="18.75" hidden="1">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="1" t="s">
         <v>130</v>
       </c>
@@ -2547,7 +2627,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="66" customHeight="1" ht="18.75" hidden="1">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66" s="1" t="s">
         <v>132</v>
       </c>
@@ -2558,7 +2638,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="67" customHeight="1" ht="18.75" hidden="1">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67" s="1" t="s">
         <v>134</v>
       </c>
@@ -2569,7 +2649,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="68" customHeight="1" ht="18.75" hidden="1">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68" s="1" t="s">
         <v>136</v>
       </c>
@@ -2580,7 +2660,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="69" customHeight="1" ht="18.75" hidden="1">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69" s="1" t="s">
         <v>138</v>
       </c>
@@ -2591,7 +2671,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="70" customHeight="1" ht="18.75" hidden="1">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70" s="1" t="s">
         <v>140</v>
       </c>
@@ -2602,7 +2682,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="71" customHeight="1" ht="18.75" hidden="1">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="1" t="s">
         <v>142</v>
       </c>
@@ -2613,7 +2693,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="72" customHeight="1" ht="18.75" hidden="1">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="1" t="s">
         <v>144</v>
       </c>
@@ -2624,7 +2704,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="73" customHeight="1" ht="18.75" hidden="1">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="1" t="s">
         <v>146</v>
       </c>
@@ -2635,7 +2715,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="74" customHeight="1" ht="18.75" hidden="1">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="1" t="s">
         <v>148</v>
       </c>
@@ -2646,7 +2726,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="75" customHeight="1" ht="18.75" hidden="1">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="1" t="s">
         <v>150</v>
       </c>
@@ -2657,7 +2737,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="76" customHeight="1" ht="18.75" hidden="1">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="1" t="s">
         <v>152</v>
       </c>
@@ -2668,7 +2748,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="77" customHeight="1" ht="18.75" hidden="1">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="1" t="s">
         <v>154</v>
       </c>
@@ -2679,7 +2759,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="78" customHeight="1" ht="18.75" hidden="1">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="1" t="s">
         <v>156</v>
       </c>
@@ -2690,7 +2770,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="79" customHeight="1" ht="18.75" hidden="1">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="1" t="s">
         <v>158</v>
       </c>
@@ -2701,7 +2781,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="80" customHeight="1" ht="18.75" hidden="1">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
         <v>160</v>
       </c>
@@ -2712,7 +2792,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="81" customHeight="1" ht="18.75" hidden="1">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81" s="1" t="s">
         <v>162</v>
       </c>
@@ -2723,7 +2803,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="82" customHeight="1" ht="18.75" hidden="1">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="1" t="s">
         <v>164</v>
       </c>
@@ -2734,7 +2814,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="83" customHeight="1" ht="18.75" hidden="1">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="1" t="s">
         <v>166</v>
       </c>
@@ -2745,7 +2825,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="84" customHeight="1" ht="18.75" hidden="1">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="1" t="s">
         <v>168</v>
       </c>
@@ -2756,7 +2836,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="85" customHeight="1" ht="18.75" hidden="1">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="1" t="s">
         <v>170</v>
       </c>
@@ -2767,7 +2847,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="86" customHeight="1" ht="18.75" hidden="1">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="1" t="s">
         <v>172</v>
       </c>
@@ -2778,7 +2858,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="87" customHeight="1" ht="18.75" hidden="1">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="1" t="s">
         <v>174</v>
       </c>
@@ -2789,7 +2869,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="88" customHeight="1" ht="18.75" hidden="1">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="1" t="s">
         <v>176</v>
       </c>
@@ -2800,7 +2880,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="89" customHeight="1" ht="18.75" hidden="1">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="1" t="s">
         <v>178</v>
       </c>
@@ -2811,7 +2891,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="90" customHeight="1" ht="18.75" hidden="1">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="1" t="s">
         <v>180</v>
       </c>
@@ -2822,7 +2902,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="91" customHeight="1" ht="18.75" hidden="1">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="1" t="s">
         <v>182</v>
       </c>
@@ -2833,7 +2913,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="92" customHeight="1" ht="18.75" hidden="1">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="1" t="s">
         <v>184</v>
       </c>
@@ -2844,7 +2924,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="93" customHeight="1" ht="18.75" hidden="1">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="1" t="s">
         <v>186</v>
       </c>
@@ -2855,7 +2935,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="94" customHeight="1" ht="18.75" hidden="1">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94" s="1" t="s">
         <v>188</v>
       </c>
@@ -2866,7 +2946,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="95" customHeight="1" ht="18.75" hidden="1">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="1" t="s">
         <v>190</v>
       </c>
@@ -2877,7 +2957,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="96" customHeight="1" ht="18.75" hidden="1">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="1" t="s">
         <v>192</v>
       </c>
@@ -2888,7 +2968,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="97" customHeight="1" ht="18.75" hidden="1">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="1" t="s">
         <v>194</v>
       </c>
@@ -2899,7 +2979,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="98" customHeight="1" ht="18.75" hidden="1">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" s="1" t="s">
         <v>196</v>
       </c>
@@ -2910,7 +2990,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="99" customHeight="1" ht="18.75" hidden="1">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A99" s="1" t="s">
         <v>198</v>
       </c>
@@ -2921,7 +3001,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="100" customHeight="1" ht="18.75" hidden="1">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A100" s="1" t="s">
         <v>200</v>
       </c>
@@ -2932,7 +3012,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="101" customHeight="1" ht="18.75" hidden="1">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" s="1" t="s">
         <v>202</v>
       </c>
@@ -2943,7 +3023,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="102" customHeight="1" ht="18.75" hidden="1">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
         <v>204</v>
       </c>
@@ -2954,7 +3034,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="103" customHeight="1" ht="18.75" hidden="1">
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" s="1" t="s">
         <v>206</v>
       </c>
@@ -2965,7 +3045,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="104" customHeight="1" ht="18.75" hidden="1">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" s="1" t="s">
         <v>208</v>
       </c>
@@ -2976,7 +3056,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="105" customHeight="1" ht="18.75" hidden="1">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" s="1" t="s">
         <v>210</v>
       </c>
@@ -2987,7 +3067,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="106" customHeight="1" ht="18.75" hidden="1">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" s="1" t="s">
         <v>212</v>
       </c>
@@ -2998,7 +3078,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="107" customHeight="1" ht="18.75" hidden="1">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" s="1" t="s">
         <v>214</v>
       </c>
@@ -3009,7 +3089,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="108" customHeight="1" ht="18.75" hidden="1">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" s="1" t="s">
         <v>216</v>
       </c>
@@ -3020,7 +3100,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="109" customHeight="1" ht="18.75" hidden="1">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" s="1" t="s">
         <v>218</v>
       </c>
@@ -3031,7 +3111,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="110" customHeight="1" ht="18.75" hidden="1">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" s="1" t="s">
         <v>220</v>
       </c>
@@ -3042,7 +3122,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="111" customHeight="1" ht="18.75" hidden="1">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" s="1" t="s">
         <v>222</v>
       </c>
@@ -3053,7 +3133,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="112" customHeight="1" ht="18.75" hidden="1">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" s="1" t="s">
         <v>224</v>
       </c>
@@ -3064,7 +3144,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="113" customHeight="1" ht="18.75" hidden="1">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" s="1" t="s">
         <v>226</v>
       </c>
@@ -3075,7 +3155,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="114" customHeight="1" ht="18.75" hidden="1">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" s="1" t="s">
         <v>228</v>
       </c>
@@ -3086,7 +3166,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="115" customHeight="1" ht="18.75" hidden="1">
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" s="1" t="s">
         <v>230</v>
       </c>
@@ -3097,7 +3177,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="116" customHeight="1" ht="18.75" hidden="1">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" s="1" t="s">
         <v>232</v>
       </c>
@@ -3108,7 +3188,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="117" customHeight="1" ht="18.75" hidden="1">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" s="1" t="s">
         <v>234</v>
       </c>
@@ -3119,7 +3199,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="118" customHeight="1" ht="18.75" hidden="1">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" s="1" t="s">
         <v>236</v>
       </c>
@@ -3130,7 +3210,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="119" customHeight="1" ht="18.75" hidden="1">
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" s="1" t="s">
         <v>238</v>
       </c>
@@ -3141,7 +3221,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="120" customHeight="1" ht="18.75" hidden="1">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" s="1" t="s">
         <v>240</v>
       </c>
@@ -3152,7 +3232,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="121" customHeight="1" ht="18.75" hidden="1">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" s="1" t="s">
         <v>242</v>
       </c>
@@ -3163,7 +3243,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="122" customHeight="1" ht="18.75" hidden="1">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" s="1" t="s">
         <v>244</v>
       </c>
@@ -3174,7 +3254,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="123" customHeight="1" ht="18.75" hidden="1">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" s="1" t="s">
         <v>246</v>
       </c>
@@ -3185,7 +3265,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="124" customHeight="1" ht="18.75" hidden="1">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
         <v>248</v>
       </c>
@@ -3196,7 +3276,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="125" customHeight="1" ht="18.75" hidden="1">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" s="1" t="s">
         <v>250</v>
       </c>
@@ -3207,7 +3287,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="126" customHeight="1" ht="18.75" hidden="1">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" s="1" t="s">
         <v>252</v>
       </c>
@@ -3218,7 +3298,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="127" customHeight="1" ht="18.75" hidden="1">
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" s="1" t="s">
         <v>254</v>
       </c>
@@ -3229,7 +3309,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="128" customHeight="1" ht="18.75" hidden="1">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" s="1" t="s">
         <v>256</v>
       </c>
@@ -3240,7 +3320,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="129" customHeight="1" ht="18.75" hidden="1">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" s="1" t="s">
         <v>258</v>
       </c>
@@ -3251,7 +3331,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="130" customHeight="1" ht="18.75" hidden="1">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" s="1" t="s">
         <v>260</v>
       </c>
@@ -3262,7 +3342,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="131" customHeight="1" ht="18.75" hidden="1">
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="1" t="s">
         <v>262</v>
       </c>
@@ -3273,7 +3353,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="132" customHeight="1" ht="18.75" hidden="1">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" s="1" t="s">
         <v>264</v>
       </c>
@@ -3284,7 +3364,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="133" customHeight="1" ht="18.75" hidden="1">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" s="1" t="s">
         <v>266</v>
       </c>
@@ -3295,7 +3375,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="134" customHeight="1" ht="18.75" hidden="1">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" s="1" t="s">
         <v>268</v>
       </c>
@@ -3306,7 +3386,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="135" customHeight="1" ht="18.75" hidden="1">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" s="1" t="s">
         <v>270</v>
       </c>
@@ -3317,7 +3397,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="136" customHeight="1" ht="18.75" hidden="1">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" s="1" t="s">
         <v>272</v>
       </c>
@@ -3328,7 +3408,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="137" customHeight="1" ht="18.75" hidden="1">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" s="1" t="s">
         <v>274</v>
       </c>
@@ -3339,7 +3419,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="138" customHeight="1" ht="18.75" hidden="1">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" s="1" t="s">
         <v>276</v>
       </c>
@@ -3350,7 +3430,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="139" customHeight="1" ht="18.75" hidden="1">
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" s="1" t="s">
         <v>278</v>
       </c>
@@ -3361,7 +3441,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="140" customHeight="1" ht="18.75" hidden="1">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" s="1" t="s">
         <v>280</v>
       </c>
@@ -3372,7 +3452,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="141" customHeight="1" ht="18.75" hidden="1">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" s="1" t="s">
         <v>282</v>
       </c>
@@ -3383,7 +3463,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="142" customHeight="1" ht="18.75" hidden="1">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" s="1" t="s">
         <v>284</v>
       </c>
@@ -3394,7 +3474,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="143" customHeight="1" ht="18.75" hidden="1">
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" s="1" t="s">
         <v>286</v>
       </c>
@@ -3405,7 +3485,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="144" customHeight="1" ht="18.75" hidden="1">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" s="1" t="s">
         <v>288</v>
       </c>
@@ -3416,7 +3496,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="145" customHeight="1" ht="18.75" hidden="1">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" s="1" t="s">
         <v>290</v>
       </c>
@@ -3427,7 +3507,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="146" customHeight="1" ht="18.75" hidden="1">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" s="1" t="s">
         <v>292</v>
       </c>
@@ -3438,7 +3518,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="147" customHeight="1" ht="18.75" hidden="1">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" s="1" t="s">
         <v>294</v>
       </c>
@@ -3449,7 +3529,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="18.75" hidden="1">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" s="1" t="s">
         <v>296</v>
       </c>
@@ -3460,7 +3540,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="18.75" hidden="1">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" s="1" t="s">
         <v>298</v>
       </c>
@@ -3471,7 +3551,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="18.75" hidden="1">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" s="1" t="s">
         <v>300</v>
       </c>
@@ -3482,7 +3562,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="18.75" hidden="1">
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" s="1" t="s">
         <v>302</v>
       </c>
@@ -3493,7 +3573,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="18.75" hidden="1">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" s="1" t="s">
         <v>304</v>
       </c>
@@ -3504,7 +3584,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="18.75" hidden="1">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" s="1" t="s">
         <v>306</v>
       </c>
@@ -3515,7 +3595,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="18.75" hidden="1">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" s="1" t="s">
         <v>308</v>
       </c>
@@ -3526,7 +3606,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="18.75" hidden="1">
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" s="1" t="s">
         <v>310</v>
       </c>
@@ -3537,7 +3617,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="18.75" hidden="1">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" s="1" t="s">
         <v>312</v>
       </c>
@@ -3548,7 +3628,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="18.75" hidden="1">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" s="1" t="s">
         <v>314</v>
       </c>
@@ -3559,7 +3639,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="18.75" hidden="1">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" s="1" t="s">
         <v>316</v>
       </c>
@@ -3570,7 +3650,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="18.75" hidden="1">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" s="1" t="s">
         <v>318</v>
       </c>
@@ -3581,7 +3661,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="18.75" hidden="1">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" s="1" t="s">
         <v>320</v>
       </c>
@@ -3592,7 +3672,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="18.75" hidden="1">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" s="1" t="s">
         <v>322</v>
       </c>
@@ -3603,7 +3683,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="18.75" hidden="1">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" s="1" t="s">
         <v>324</v>
       </c>
@@ -3614,7 +3694,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="18.75" hidden="1">
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" s="1" t="s">
         <v>326</v>
       </c>
@@ -3625,7 +3705,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="18.75" hidden="1">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" s="1" t="s">
         <v>328</v>
       </c>
@@ -3636,7 +3716,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="18.75" hidden="1">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" s="1" t="s">
         <v>330</v>
       </c>
@@ -3647,7 +3727,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="18.75" hidden="1">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" s="1" t="s">
         <v>332</v>
       </c>
@@ -3658,7 +3738,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="167" customHeight="1" ht="18.75" hidden="1">
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" s="1" t="s">
         <v>334</v>
       </c>
@@ -3669,7 +3749,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="18.75" hidden="1">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" s="1" t="s">
         <v>336</v>
       </c>
@@ -3680,7 +3760,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="18.75" hidden="1">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" s="1" t="s">
         <v>338</v>
       </c>
@@ -3691,7 +3771,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="18.75" hidden="1">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" s="1" t="s">
         <v>340</v>
       </c>
@@ -3702,7 +3782,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="171" customHeight="1" ht="18.75" hidden="1">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" s="1" t="s">
         <v>342</v>
       </c>
@@ -3713,7 +3793,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="18.75" hidden="1">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" s="1" t="s">
         <v>344</v>
       </c>
@@ -3724,7 +3804,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="18.75" hidden="1">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" s="1" t="s">
         <v>346</v>
       </c>
@@ -3735,7 +3815,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="18.75" hidden="1">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" s="1" t="s">
         <v>348</v>
       </c>
@@ -3746,7 +3826,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="18.75" hidden="1">
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" s="1" t="s">
         <v>350</v>
       </c>
@@ -3757,7 +3837,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="18.75" hidden="1">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" s="1" t="s">
         <v>352</v>
       </c>
@@ -3768,7 +3848,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="18.75" hidden="1">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="1" t="s">
         <v>354</v>
       </c>
@@ -3779,7 +3859,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="18.75" hidden="1">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="1" t="s">
         <v>356</v>
       </c>
@@ -3790,7 +3870,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="18.75" hidden="1">
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="1" t="s">
         <v>358</v>
       </c>
@@ -3801,7 +3881,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="180" customHeight="1" ht="18.75" hidden="1">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="1" t="s">
         <v>360</v>
       </c>
@@ -3812,7 +3892,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="181" customHeight="1" ht="18.75" hidden="1">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="1" t="s">
         <v>362</v>
       </c>
@@ -3823,7 +3903,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="182" customHeight="1" ht="18.75" hidden="1">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="1" t="s">
         <v>364</v>
       </c>
@@ -3834,7 +3914,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="183" customHeight="1" ht="18.75" hidden="1">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="1" t="s">
         <v>366</v>
       </c>
@@ -3845,7 +3925,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="184" customHeight="1" ht="18.75" hidden="1">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="1" t="s">
         <v>368</v>
       </c>
@@ -3856,7 +3936,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="185" customHeight="1" ht="18.75" hidden="1">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="1" t="s">
         <v>370</v>
       </c>
@@ -3867,7 +3947,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="186" customHeight="1" ht="18.75" hidden="1">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="1" t="s">
         <v>372</v>
       </c>
@@ -3878,7 +3958,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="187" customHeight="1" ht="18.75" hidden="1">
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="1" t="s">
         <v>374</v>
       </c>
@@ -3889,7 +3969,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="188" customHeight="1" ht="18.75" hidden="1">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="1" t="s">
         <v>376</v>
       </c>
@@ -3900,7 +3980,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="189" customHeight="1" ht="18.75" hidden="1">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="1" t="s">
         <v>378</v>
       </c>
@@ -3911,7 +3991,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="190" customHeight="1" ht="18.75" hidden="1">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="1" t="s">
         <v>380</v>
       </c>
@@ -3922,7 +4002,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="191" customHeight="1" ht="18.75" hidden="1">
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="1" t="s">
         <v>382</v>
       </c>
@@ -3933,7 +4013,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="192" customHeight="1" ht="18.75" hidden="1">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="1" t="s">
         <v>384</v>
       </c>
@@ -3944,7 +4024,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="193" customHeight="1" ht="18.75" hidden="1">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="1" t="s">
         <v>386</v>
       </c>
@@ -3955,7 +4035,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="194" customHeight="1" ht="18.75" hidden="1">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" s="1" t="s">
         <v>388</v>
       </c>
@@ -3966,7 +4046,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="195" customHeight="1" ht="18.75" hidden="1">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="1" t="s">
         <v>390</v>
       </c>
@@ -3977,7 +4057,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="196" customHeight="1" ht="18.75" hidden="1">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="1" t="s">
         <v>392</v>
       </c>
@@ -3988,7 +4068,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="197" customHeight="1" ht="18.75" hidden="1">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="1" t="s">
         <v>394</v>
       </c>
@@ -3999,7 +4079,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="198" customHeight="1" ht="18.75" hidden="1">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="1" t="s">
         <v>396</v>
       </c>
@@ -4010,7 +4090,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="199" customHeight="1" ht="18.75" hidden="1">
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="1" t="s">
         <v>398</v>
       </c>
@@ -4021,7 +4101,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="200" customHeight="1" ht="18.75" hidden="1">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="1" t="s">
         <v>400</v>
       </c>
@@ -4032,7 +4112,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="201" customHeight="1" ht="18.75" hidden="1">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="1" t="s">
         <v>402</v>
       </c>
@@ -4043,7 +4123,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="202" customHeight="1" ht="18.75" hidden="1">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A202" s="1" t="s">
         <v>404</v>
       </c>
@@ -4054,7 +4134,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="203" customHeight="1" ht="18.75" hidden="1">
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A203" s="1" t="s">
         <v>406</v>
       </c>
@@ -4065,7 +4145,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="204" customHeight="1" ht="18.75" hidden="1">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A204" s="1" t="s">
         <v>408</v>
       </c>
@@ -4076,7 +4156,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="205" customHeight="1" ht="18.75" hidden="1">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A205" s="1" t="s">
         <v>410</v>
       </c>
@@ -4087,7 +4167,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="206" customHeight="1" ht="18.75" hidden="1">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A206" s="1" t="s">
         <v>412</v>
       </c>
@@ -4098,7 +4178,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="207" customHeight="1" ht="18.75" hidden="1">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A207" s="1" t="s">
         <v>414</v>
       </c>
@@ -4109,7 +4189,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="208" customHeight="1" ht="18.75" hidden="1">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A208" s="1" t="s">
         <v>416</v>
       </c>
@@ -4120,7 +4200,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="209" customHeight="1" ht="18.75" hidden="1">
+    <row r="209" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A209" s="1" t="s">
         <v>418</v>
       </c>
@@ -4131,7 +4211,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="210" customHeight="1" ht="18.75" hidden="1">
+    <row r="210" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A210" s="1" t="s">
         <v>420</v>
       </c>
@@ -4142,7 +4222,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="211" customHeight="1" ht="18.75" hidden="1">
+    <row r="211" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A211" s="1" t="s">
         <v>422</v>
       </c>
@@ -4153,7 +4233,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="212" customHeight="1" ht="18.75" hidden="1">
+    <row r="212" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A212" s="1" t="s">
         <v>424</v>
       </c>
@@ -4164,7 +4244,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="213" customHeight="1" ht="18.75" hidden="1">
+    <row r="213" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A213" s="1" t="s">
         <v>426</v>
       </c>
@@ -4175,7 +4255,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="214" customHeight="1" ht="18.75" hidden="1">
+    <row r="214" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A214" s="1" t="s">
         <v>428</v>
       </c>
@@ -4186,7 +4266,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="215" customHeight="1" ht="18.75" hidden="1">
+    <row r="215" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A215" s="1" t="s">
         <v>430</v>
       </c>
@@ -4197,7 +4277,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="216" customHeight="1" ht="18.75" hidden="1">
+    <row r="216" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A216" s="1" t="s">
         <v>432</v>
       </c>
@@ -4208,7 +4288,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="217" customHeight="1" ht="18.75" hidden="1">
+    <row r="217" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A217" s="1" t="s">
         <v>434</v>
       </c>
@@ -4219,7 +4299,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="218" customHeight="1" ht="18.75" hidden="1">
+    <row r="218" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A218" s="1" t="s">
         <v>436</v>
       </c>
@@ -4230,7 +4310,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="219" customHeight="1" ht="18.75" hidden="1">
+    <row r="219" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A219" s="1" t="s">
         <v>438</v>
       </c>
@@ -4241,7 +4321,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="220" customHeight="1" ht="18.75" hidden="1">
+    <row r="220" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A220" s="1" t="s">
         <v>440</v>
       </c>
@@ -4252,7 +4332,7 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="221" customHeight="1" ht="18.75" hidden="1">
+    <row r="221" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A221" s="1" t="s">
         <v>442</v>
       </c>
@@ -4263,128 +4343,260 @@
         <v>5</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="222" customHeight="1" ht="18.75" customFormat="1" s="3" hidden="1">
+    <row r="222" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A222" s="4" t="s">
         <v>444</v>
       </c>
-      <c r="B222" s="5" t="s">
+      <c r="B222" s="7" t="s">
         <v>445</v>
       </c>
       <c r="C222" s="4" t="s">
         <v>446</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="223" customHeight="1" ht="18.75" customFormat="1" s="3" hidden="1">
+    <row r="223" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A223" s="4" t="s">
         <v>447</v>
       </c>
-      <c r="B223" s="5" t="s">
+      <c r="B223" s="7" t="s">
         <v>448</v>
       </c>
       <c r="C223" s="4" t="s">
         <v>446</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="224" customHeight="1" ht="18.75" customFormat="1" s="3" hidden="1">
+    <row r="224" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A224" s="4" t="s">
         <v>449</v>
       </c>
-      <c r="B224" s="5" t="s">
+      <c r="B224" s="7" t="s">
         <v>450</v>
       </c>
       <c r="C224" s="4" t="s">
         <v>446</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="225" customHeight="1" ht="18.75" customFormat="1" s="3" hidden="1">
+    <row r="225" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A225" s="4" t="s">
         <v>451</v>
       </c>
-      <c r="B225" s="5" t="s">
+      <c r="B225" s="7" t="s">
         <v>452</v>
       </c>
       <c r="C225" s="4" t="s">
         <v>446</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="226" customHeight="1" ht="18.75" customFormat="1" s="3" hidden="1">
+    <row r="226" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A226" s="4" t="s">
         <v>453</v>
       </c>
-      <c r="B226" s="5" t="s">
+      <c r="B226" s="7" t="s">
         <v>454</v>
       </c>
       <c r="C226" s="4" t="s">
         <v>446</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="227" customHeight="1" ht="18.75" customFormat="1" s="3" hidden="1">
+    <row r="227" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A227" s="4" t="s">
         <v>455</v>
       </c>
-      <c r="B227" s="5" t="s">
+      <c r="B227" s="7" t="s">
         <v>456</v>
       </c>
       <c r="C227" s="4" t="s">
         <v>457</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="228" customHeight="1" ht="18.75" customFormat="1" s="3" hidden="1">
+    <row r="228" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A228" s="4" t="s">
         <v>458</v>
       </c>
-      <c r="B228" s="5" t="s">
+      <c r="B228" s="7" t="s">
         <v>459</v>
       </c>
       <c r="C228" s="4" t="s">
         <v>457</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="229" customHeight="1" ht="18.75" customFormat="1" s="3" hidden="1">
+    <row r="229" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A229" s="4" t="s">
         <v>460</v>
       </c>
-      <c r="B229" s="5" t="s">
+      <c r="B229" s="7" t="s">
         <v>461</v>
       </c>
       <c r="C229" s="4" t="s">
         <v>457</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="230" customHeight="1" ht="18.75" customFormat="1" s="3" hidden="1">
+    <row r="230" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A230" s="4" t="s">
         <v>462</v>
       </c>
-      <c r="B230" s="5" t="s">
+      <c r="B230" s="7" t="s">
         <v>463</v>
       </c>
       <c r="C230" s="4" t="s">
         <v>464</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="231" customHeight="1" ht="18.75" customFormat="1" s="3" hidden="1">
+    <row r="231" spans="1:3" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A231" s="4" t="s">
         <v>465</v>
       </c>
-      <c r="B231" s="5" t="s">
+      <c r="B231" s="7" t="s">
         <v>466</v>
       </c>
       <c r="C231" s="4" t="s">
         <v>464</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="232" customHeight="1" ht="18.75" customFormat="1" s="3" hidden="1">
+    <row r="232" spans="1:3" s="3" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A232" s="4" t="s">
         <v>467</v>
       </c>
-      <c r="B232" s="5" t="s">
+      <c r="B232" s="7" t="s">
         <v>468</v>
       </c>
       <c r="C232" s="4" t="s">
         <v>464</v>
       </c>
     </row>
+    <row r="233" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A233" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="B233" s="6" t="s">
+        <v>470</v>
+      </c>
+      <c r="C233" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="234" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A234" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="B234" s="6" t="s">
+        <v>472</v>
+      </c>
+      <c r="C234" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="235" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A235" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="B235" s="6" t="s">
+        <v>474</v>
+      </c>
+      <c r="C235" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="236" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A236" s="5" t="s">
+        <v>475</v>
+      </c>
+      <c r="B236" s="6" t="s">
+        <v>476</v>
+      </c>
+      <c r="C236" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="237" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A237" s="5" t="s">
+        <v>477</v>
+      </c>
+      <c r="B237" s="6" t="s">
+        <v>478</v>
+      </c>
+      <c r="C237" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="238" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A238" s="5" t="s">
+        <v>479</v>
+      </c>
+      <c r="B238" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="C238" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="239" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A239" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="B239" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="C239" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="240" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A240" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="B240" s="6" t="s">
+        <v>483</v>
+      </c>
+      <c r="C240" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="241" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A241" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="B241" s="6" t="s">
+        <v>485</v>
+      </c>
+      <c r="C241" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="242" spans="1:3" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A242" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="B242" s="6" t="s">
+        <v>487</v>
+      </c>
+      <c r="C242" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B233" r:id="rId1" xr:uid="{B554C6EE-FFDF-48A1-9376-EC9DC31A6359}"/>
+    <hyperlink ref="B234" r:id="rId2" xr:uid="{C36C5949-97C7-472D-ABC8-5CDCF6749F36}"/>
+    <hyperlink ref="B235" r:id="rId3" xr:uid="{659F1303-944D-426E-8C9F-B4B12A78E2A6}"/>
+    <hyperlink ref="B236" r:id="rId4" xr:uid="{3063DB71-821C-4818-B505-E6FCF6166AB0}"/>
+    <hyperlink ref="B237" r:id="rId5" xr:uid="{84397185-FF3C-427E-9FDC-F40C64AE2DAC}"/>
+    <hyperlink ref="B239" r:id="rId6" xr:uid="{EEB52FAB-3C9F-4F19-9259-68A9073A368E}"/>
+    <hyperlink ref="B240" r:id="rId7" xr:uid="{E3780798-7655-4138-B67C-BEAED848D7A3}"/>
+    <hyperlink ref="B241" r:id="rId8" xr:uid="{B3A183BC-E3B9-4592-836D-2C8758D34FAD}"/>
+    <hyperlink ref="B242" r:id="rId9" xr:uid="{D608081A-9432-4469-9B2C-2DF217C04AF9}"/>
+    <hyperlink ref="B224" r:id="rId10" xr:uid="{0AB7F051-47B2-4E61-A973-53AC2B970965}"/>
+    <hyperlink ref="B228" r:id="rId11" xr:uid="{01346ED6-3785-4A00-8F96-4AA2811C88A1}"/>
+    <hyperlink ref="B227" r:id="rId12" xr:uid="{1321C569-ACED-4E1A-B568-A559F11ECF05}"/>
+    <hyperlink ref="B226" r:id="rId13" xr:uid="{9C7D8DE3-8FB1-43E5-AF2A-0AA28CEB95F6}"/>
+    <hyperlink ref="B222" r:id="rId14" xr:uid="{E3AAA498-51F0-429A-A13F-62405D5E8BCB}"/>
+    <hyperlink ref="B223" r:id="rId15" xr:uid="{7A6EAE2C-C753-40AD-8035-94D929D4ACCA}"/>
+    <hyperlink ref="B225" r:id="rId16" xr:uid="{C7F25E51-5FE1-41D4-98E3-B43179F4947D}"/>
+    <hyperlink ref="B229" r:id="rId17" xr:uid="{EFD4B0CC-DAC6-4CDF-8548-1B1E94BBDE6B}"/>
+    <hyperlink ref="B230" r:id="rId18" xr:uid="{E5B22229-9AE4-4F36-BEB9-AE9942ADD16B}"/>
+    <hyperlink ref="B231" r:id="rId19" xr:uid="{FB54459F-B8A0-4D14-BB69-15559BFECCCB}"/>
+    <hyperlink ref="B232" r:id="rId20" xr:uid="{107C064A-D46B-4982-A325-123FBE2239E8}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>